<commit_message>
New output tables with bad BESE removed.
</commit_message>
<xml_diff>
--- a/output_tables/group_summary.xlsx
+++ b/output_tables/group_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{A6B92D8E-5CB2-4AA8-94ED-0214DE4A4096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{608BF0BB-7FAA-44B2-AEEF-B8F78EEBCE87}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{59E47FFB-B8F7-45C3-A319-0743BC9995C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF9EF313-13FD-43B7-83F0-2D6B6F9A5433}"/>
   <bookViews>
-    <workbookView xWindow="165" yWindow="90" windowWidth="28635" windowHeight="15390" xr2:uid="{0DC45B1B-F6FD-42B0-BE43-E76595711F53}"/>
+    <workbookView xWindow="1560" yWindow="240" windowWidth="24405" windowHeight="15390" xr2:uid="{DE4F24FA-FBA3-478C-9F9E-E001BBB69A88}"/>
   </bookViews>
   <sheets>
     <sheet name="group_summary" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="206">
   <si>
     <t>group_no</t>
   </si>
@@ -31,24 +31,36 @@
     <t>method</t>
   </si>
   <si>
+    <t>donorsites</t>
+  </si>
+  <si>
     <t>AMS_shallow</t>
   </si>
   <si>
     <t>staple</t>
   </si>
   <si>
+    <t>Thompson Cove</t>
+  </si>
+  <si>
     <t>AMS_deep</t>
   </si>
   <si>
     <t>AND_west1</t>
   </si>
   <si>
+    <t>Ketron Island</t>
+  </si>
+  <si>
     <t>AND_west2</t>
   </si>
   <si>
     <t>rebar</t>
   </si>
   <si>
+    <t>Sandy Point</t>
+  </si>
+  <si>
     <t>AND_south1</t>
   </si>
   <si>
@@ -58,6 +70,9 @@
     <t>turf</t>
   </si>
   <si>
+    <t>Rocky Bay</t>
+  </si>
+  <si>
     <t>AND_south_L1</t>
   </si>
   <si>
@@ -73,6 +88,9 @@
     <t>AMS_deeper</t>
   </si>
   <si>
+    <t>Anderson Island</t>
+  </si>
+  <si>
     <t>AND_west3</t>
   </si>
   <si>
@@ -82,6 +100,9 @@
     <t>AND_west4</t>
   </si>
   <si>
+    <t>DuPont Wharf</t>
+  </si>
+  <si>
     <t>AND_west5</t>
   </si>
   <si>
@@ -94,9 +115,27 @@
     <t>BB_test_1</t>
   </si>
   <si>
+    <t>Dumas Bay</t>
+  </si>
+  <si>
+    <t>Fay Bainbridge</t>
+  </si>
+  <si>
+    <t>Henry Island</t>
+  </si>
+  <si>
+    <t>Ship Harbor</t>
+  </si>
+  <si>
+    <t>Mixed</t>
+  </si>
+  <si>
     <t>CHC</t>
   </si>
   <si>
+    <t>Creosote Point</t>
+  </si>
+  <si>
     <t>COM_shallow</t>
   </si>
   <si>
@@ -118,6 +157,9 @@
     <t>burlap</t>
   </si>
   <si>
+    <t>Cutts Island</t>
+  </si>
+  <si>
     <t>DEL_P1</t>
   </si>
   <si>
@@ -136,6 +178,9 @@
     <t>DEL_L</t>
   </si>
   <si>
+    <t>Green Point</t>
+  </si>
+  <si>
     <t>DEL_west_shallow_1</t>
   </si>
   <si>
@@ -157,6 +202,9 @@
     <t>ELD_shallow</t>
   </si>
   <si>
+    <t>Windy Bluff</t>
+  </si>
+  <si>
     <t>ELD_deep</t>
   </si>
   <si>
@@ -166,6 +214,9 @@
     <t>ELW_deep_west</t>
   </si>
   <si>
+    <t>Freshwater Bay</t>
+  </si>
+  <si>
     <t>ELW_shallow_west</t>
   </si>
   <si>
@@ -199,12 +250,18 @@
     <t>HAR_deep_L1</t>
   </si>
   <si>
+    <t>Rocky Point</t>
+  </si>
+  <si>
     <t>HAR_shallow_L1</t>
   </si>
   <si>
     <t>HAR_shallow_L2</t>
   </si>
   <si>
+    <t>Anderson Island, Windy Bluff</t>
+  </si>
+  <si>
     <t>HAR_shallow_L3</t>
   </si>
   <si>
@@ -229,12 +286,18 @@
     <t>JSP_mid_shallow</t>
   </si>
   <si>
+    <t>Windy Bluff/Thompson Cove</t>
+  </si>
+  <si>
     <t>JSP_mid_deep</t>
   </si>
   <si>
     <t>JSP_mid_south_P1</t>
   </si>
   <si>
+    <t>Windy Bluff and Thompson Cove</t>
+  </si>
+  <si>
     <t>JSP_mid_north_P1</t>
   </si>
   <si>
@@ -319,6 +382,9 @@
     <t>LBT_east</t>
   </si>
   <si>
+    <t>Sandy Hook</t>
+  </si>
+  <si>
     <t>LBT_west</t>
   </si>
   <si>
@@ -388,6 +454,9 @@
     <t>PTG_5</t>
   </si>
   <si>
+    <t>Point Julia</t>
+  </si>
+  <si>
     <t>PTG_2</t>
   </si>
   <si>
@@ -451,6 +520,9 @@
     <t>QLC01</t>
   </si>
   <si>
+    <t>Quilcene Bay</t>
+  </si>
+  <si>
     <t>QLC_north1</t>
   </si>
   <si>
@@ -481,9 +553,15 @@
     <t>SHB_1</t>
   </si>
   <si>
+    <t>Shine Beach</t>
+  </si>
+  <si>
     <t>SKG_1</t>
   </si>
   <si>
+    <t>Skagit Bay</t>
+  </si>
+  <si>
     <t>SKG_2</t>
   </si>
   <si>
@@ -502,18 +580,30 @@
     <t>WES_east</t>
   </si>
   <si>
+    <t>PNNL - MSL Tanks</t>
+  </si>
+  <si>
     <t>WES_west</t>
   </si>
   <si>
     <t>WES_A</t>
   </si>
   <si>
+    <t>Bell Point, Stuart Island</t>
+  </si>
+  <si>
     <t>WES_B</t>
   </si>
   <si>
+    <t>Bell Point</t>
+  </si>
+  <si>
     <t>WES_C</t>
   </si>
   <si>
+    <t>Mitchell Bay</t>
+  </si>
+  <si>
     <t>WES_D</t>
   </si>
   <si>
@@ -535,7 +625,19 @@
     <t>ZAN_4</t>
   </si>
   <si>
-    <t>ok. Multiple plantings at this loc_code.</t>
+    <t>Is the 'mix' specifically drawn from the other test cases at BB_test_1?</t>
+  </si>
+  <si>
+    <t>needs resolution - a 4-record polygon planting with different method for each corner; "drop"</t>
+  </si>
+  <si>
+    <t>needs resolution - a 4-record polygon planting with different method for each corner; "retain"</t>
+  </si>
+  <si>
+    <t>BESE case - needs to be addressed somehow. Activity filter gives multiple BESE planting locations as one group, but these are distinct in location and coords.</t>
+  </si>
+  <si>
+    <t>Is this a mix of donor plants from the other co-located cases?</t>
   </si>
 </sst>
 </file>
@@ -860,7 +962,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.749992370372631"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1424,18 +1526,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125E202D-C6A1-4C20-9FAE-C33475A4CD5A}">
-  <dimension ref="A1:E197"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4FED8F-716B-4B06-A141-CFC261A1ADE2}">
+  <dimension ref="A1:F196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.140625" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="106.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1445,8 +1548,11 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1454,13 +1560,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1468,13 +1577,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1482,13 +1594,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1496,13 +1611,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1510,13 +1628,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1524,13 +1645,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1538,13 +1662,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1552,13 +1679,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1566,13 +1696,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1580,13 +1713,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1594,13 +1730,16 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1608,13 +1747,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1622,13 +1764,16 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1636,13 +1781,16 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1650,13 +1798,16 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1664,13 +1815,16 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1678,13 +1832,16 @@
         <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1692,13 +1849,16 @@
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1706,13 +1866,16 @@
         <v>19</v>
       </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1720,13 +1883,16 @@
         <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1734,13 +1900,16 @@
         <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1748,13 +1917,19 @@
         <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1762,13 +1937,16 @@
         <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D24" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1776,13 +1954,16 @@
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="D25" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1790,13 +1971,16 @@
         <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1804,13 +1988,16 @@
         <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="D27" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1818,13 +2005,16 @@
         <v>27</v>
       </c>
       <c r="C28" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1832,13 +2022,16 @@
         <v>28</v>
       </c>
       <c r="C29" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D29" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1846,13 +2039,16 @@
         <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D30" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E30" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1860,13 +2056,16 @@
         <v>30</v>
       </c>
       <c r="C31" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1874,13 +2073,16 @@
         <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="D32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1888,13 +2090,16 @@
         <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D33" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E33" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1902,13 +2107,16 @@
         <v>33</v>
       </c>
       <c r="C34" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D34" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1916,13 +2124,16 @@
         <v>34</v>
       </c>
       <c r="C35" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="D35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1930,13 +2141,16 @@
         <v>35</v>
       </c>
       <c r="C36" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="D36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1944,13 +2158,16 @@
         <v>36</v>
       </c>
       <c r="C37" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="D37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1958,13 +2175,16 @@
         <v>37</v>
       </c>
       <c r="C38" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="D38" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1972,13 +2192,16 @@
         <v>38</v>
       </c>
       <c r="C39" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1986,13 +2209,16 @@
         <v>39</v>
       </c>
       <c r="C40" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="D40" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2000,13 +2226,16 @@
         <v>40</v>
       </c>
       <c r="C41" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D41" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2014,13 +2243,16 @@
         <v>41</v>
       </c>
       <c r="C42" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2028,13 +2260,16 @@
         <v>42</v>
       </c>
       <c r="C43" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2042,13 +2277,16 @@
         <v>43</v>
       </c>
       <c r="C44" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2056,13 +2294,16 @@
         <v>44</v>
       </c>
       <c r="C45" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2070,13 +2311,16 @@
         <v>45</v>
       </c>
       <c r="C46" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2084,13 +2328,16 @@
         <v>46</v>
       </c>
       <c r="C47" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="D47" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2098,13 +2345,16 @@
         <v>47</v>
       </c>
       <c r="C48" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="D48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E48" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2112,13 +2362,16 @@
         <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="D49" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E49" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2126,13 +2379,16 @@
         <v>49</v>
       </c>
       <c r="C50" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2140,13 +2396,16 @@
         <v>50</v>
       </c>
       <c r="C51" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="D51" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2154,13 +2413,16 @@
         <v>51</v>
       </c>
       <c r="C52" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="D52" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2168,13 +2430,16 @@
         <v>52</v>
       </c>
       <c r="C53" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="D53" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2182,13 +2447,16 @@
         <v>53</v>
       </c>
       <c r="C54" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D54" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2196,13 +2464,16 @@
         <v>54</v>
       </c>
       <c r="C55" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D55" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E55" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2210,13 +2481,16 @@
         <v>55</v>
       </c>
       <c r="C56" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D56" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2224,13 +2498,16 @@
         <v>56</v>
       </c>
       <c r="C57" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D57" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2238,13 +2515,16 @@
         <v>57</v>
       </c>
       <c r="C58" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="D58" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E58" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2252,13 +2532,16 @@
         <v>58</v>
       </c>
       <c r="C59" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="D59" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2266,13 +2549,16 @@
         <v>59</v>
       </c>
       <c r="C60" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D60" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2280,13 +2566,16 @@
         <v>60</v>
       </c>
       <c r="C61" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="D61" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2294,13 +2583,16 @@
         <v>61</v>
       </c>
       <c r="C62" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="D62" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E62" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2308,13 +2600,16 @@
         <v>62</v>
       </c>
       <c r="C63" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="D63" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2322,13 +2617,16 @@
         <v>63</v>
       </c>
       <c r="C64" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D64" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2336,13 +2634,16 @@
         <v>64</v>
       </c>
       <c r="C65" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="D65" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2350,13 +2651,16 @@
         <v>65</v>
       </c>
       <c r="C66" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="D66" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E66" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2364,13 +2668,16 @@
         <v>66</v>
       </c>
       <c r="C67" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="D67" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2378,13 +2685,16 @@
         <v>67</v>
       </c>
       <c r="C68" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="D68" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2392,13 +2702,16 @@
         <v>68</v>
       </c>
       <c r="C69" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="D69" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E69" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2406,13 +2719,16 @@
         <v>69</v>
       </c>
       <c r="C70" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="D70" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2420,13 +2736,16 @@
         <v>70</v>
       </c>
       <c r="C71" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="D71" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E71" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2434,13 +2753,16 @@
         <v>71</v>
       </c>
       <c r="C72" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="D72" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E72" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2448,13 +2770,16 @@
         <v>72</v>
       </c>
       <c r="C73" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="D73" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E73" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2462,13 +2787,16 @@
         <v>73</v>
       </c>
       <c r="C74" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="D74" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2476,13 +2804,16 @@
         <v>74</v>
       </c>
       <c r="C75" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="D75" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E75" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2490,13 +2821,16 @@
         <v>75</v>
       </c>
       <c r="C76" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="D76" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2504,13 +2838,16 @@
         <v>76</v>
       </c>
       <c r="C77" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D77" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2518,13 +2855,16 @@
         <v>77</v>
       </c>
       <c r="C78" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2532,13 +2872,16 @@
         <v>78</v>
       </c>
       <c r="C79" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2546,13 +2889,16 @@
         <v>79</v>
       </c>
       <c r="C80" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="D80" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2560,13 +2906,16 @@
         <v>80</v>
       </c>
       <c r="C81" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="D81" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E81" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2574,13 +2923,16 @@
         <v>81</v>
       </c>
       <c r="C82" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="D82" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E82" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2588,13 +2940,16 @@
         <v>82</v>
       </c>
       <c r="C83" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="D83" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2602,13 +2957,16 @@
         <v>83</v>
       </c>
       <c r="C84" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="D84" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E84" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2616,13 +2974,16 @@
         <v>84</v>
       </c>
       <c r="C85" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="D85" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E85" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2630,13 +2991,16 @@
         <v>85</v>
       </c>
       <c r="C86" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="D86" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E86" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2644,13 +3008,16 @@
         <v>86</v>
       </c>
       <c r="C87" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="D87" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E87" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2658,27 +3025,36 @@
         <v>87</v>
       </c>
       <c r="C88" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="D88" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E88" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89">
         <v>88</v>
       </c>
-      <c r="C89" t="s">
-        <v>81</v>
+      <c r="C89" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="D89" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E89" t="s">
+        <v>26</v>
+      </c>
+      <c r="F89" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2686,16 +3062,19 @@
         <v>89</v>
       </c>
       <c r="C90" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="E90" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="F90" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2703,13 +3082,19 @@
         <v>90</v>
       </c>
       <c r="C91" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+      <c r="E91" t="s">
+        <v>26</v>
+      </c>
+      <c r="F91" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2717,13 +3102,19 @@
         <v>91</v>
       </c>
       <c r="C92" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+      <c r="E92" t="s">
+        <v>26</v>
+      </c>
+      <c r="F92" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2731,13 +3122,16 @@
         <v>92</v>
       </c>
       <c r="C93" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="D93" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E93" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2745,13 +3139,16 @@
         <v>93</v>
       </c>
       <c r="C94" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="D94" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E94" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2759,13 +3156,16 @@
         <v>94</v>
       </c>
       <c r="C95" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="D95" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E95" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2773,13 +3173,16 @@
         <v>95</v>
       </c>
       <c r="C96" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="D96" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E96" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2787,13 +3190,16 @@
         <v>96</v>
       </c>
       <c r="C97" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="D97" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E97" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2801,13 +3207,16 @@
         <v>97</v>
       </c>
       <c r="C98" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="D98" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E98" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2815,13 +3224,16 @@
         <v>98</v>
       </c>
       <c r="C99" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="D99" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E99" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2829,13 +3241,16 @@
         <v>99</v>
       </c>
       <c r="C100" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="D100" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E100" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2843,13 +3258,16 @@
         <v>100</v>
       </c>
       <c r="C101" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="D101" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E101" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -2857,13 +3275,16 @@
         <v>101</v>
       </c>
       <c r="C102" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="D102" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E102" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -2871,13 +3292,16 @@
         <v>102</v>
       </c>
       <c r="C103" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="D103" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E103" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -2885,13 +3309,16 @@
         <v>103</v>
       </c>
       <c r="C104" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D104" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E104" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -2899,13 +3326,16 @@
         <v>104</v>
       </c>
       <c r="C105" t="s">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="D105" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E105" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -2913,13 +3343,16 @@
         <v>105</v>
       </c>
       <c r="C106" t="s">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="D106" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E106" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -2927,13 +3360,16 @@
         <v>106</v>
       </c>
       <c r="C107" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="D107" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E107" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -2941,13 +3377,16 @@
         <v>107</v>
       </c>
       <c r="C108" t="s">
-        <v>93</v>
+        <v>115</v>
       </c>
       <c r="D108" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E108" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -2955,13 +3394,16 @@
         <v>108</v>
       </c>
       <c r="C109" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="D109" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E109" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -2969,13 +3411,16 @@
         <v>109</v>
       </c>
       <c r="C110" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="D110" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E110" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -2983,13 +3428,16 @@
         <v>110</v>
       </c>
       <c r="C111" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="D111" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E111" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -2997,13 +3445,16 @@
         <v>111</v>
       </c>
       <c r="C112" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="D112" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E112" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3011,13 +3462,16 @@
         <v>112</v>
       </c>
       <c r="C113" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="D113" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E113" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3025,13 +3479,16 @@
         <v>113</v>
       </c>
       <c r="C114" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="D114" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E114" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3039,13 +3496,16 @@
         <v>114</v>
       </c>
       <c r="C115" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D115" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E115" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3053,13 +3513,16 @@
         <v>115</v>
       </c>
       <c r="C116" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="D116" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E116" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3067,13 +3530,16 @@
         <v>116</v>
       </c>
       <c r="C117" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="D117" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E117" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3081,13 +3547,16 @@
         <v>117</v>
       </c>
       <c r="C118" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D118" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E118" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -3095,13 +3564,16 @@
         <v>118</v>
       </c>
       <c r="C119" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="D119" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E119" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -3109,13 +3581,16 @@
         <v>119</v>
       </c>
       <c r="C120" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="D120" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E120" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -3123,13 +3598,16 @@
         <v>120</v>
       </c>
       <c r="C121" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="D121" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E121" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3137,13 +3615,16 @@
         <v>121</v>
       </c>
       <c r="C122" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="D122" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E122" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3151,13 +3632,16 @@
         <v>122</v>
       </c>
       <c r="C123" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="D123" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E123" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3165,13 +3649,16 @@
         <v>123</v>
       </c>
       <c r="C124" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D124" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E124" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3179,13 +3666,16 @@
         <v>124</v>
       </c>
       <c r="C125" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="D125" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E125" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3193,13 +3683,16 @@
         <v>125</v>
       </c>
       <c r="C126" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="D126" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E126" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3207,13 +3700,16 @@
         <v>126</v>
       </c>
       <c r="C127" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="D127" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E127" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3221,13 +3717,16 @@
         <v>127</v>
       </c>
       <c r="C128" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="D128" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E128" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3235,13 +3734,16 @@
         <v>128</v>
       </c>
       <c r="C129" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="D129" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E129" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3249,13 +3751,16 @@
         <v>129</v>
       </c>
       <c r="C130" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="D130" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E130" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3263,13 +3768,16 @@
         <v>130</v>
       </c>
       <c r="C131" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="D131" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E131" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -3277,13 +3785,16 @@
         <v>131</v>
       </c>
       <c r="C132" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="D132" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E132" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -3291,13 +3802,16 @@
         <v>132</v>
       </c>
       <c r="C133" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="D133" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E133" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -3305,13 +3819,16 @@
         <v>133</v>
       </c>
       <c r="C134" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="D134" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E134" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -3319,13 +3836,16 @@
         <v>134</v>
       </c>
       <c r="C135" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="D135" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E135" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -3333,13 +3853,16 @@
         <v>135</v>
       </c>
       <c r="C136" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="D136" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E136" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -3347,13 +3870,16 @@
         <v>136</v>
       </c>
       <c r="C137" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="D137" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E137" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -3361,13 +3887,16 @@
         <v>137</v>
       </c>
       <c r="C138" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="D138" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E138" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
@@ -3375,13 +3904,16 @@
         <v>138</v>
       </c>
       <c r="C139" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="D139" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E139" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
@@ -3389,13 +3921,16 @@
         <v>139</v>
       </c>
       <c r="C140" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="D140" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E140" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
@@ -3403,13 +3938,16 @@
         <v>140</v>
       </c>
       <c r="C141" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="D141" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E141" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
@@ -3417,13 +3955,16 @@
         <v>141</v>
       </c>
       <c r="C142" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="D142" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E142" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -3431,13 +3972,16 @@
         <v>142</v>
       </c>
       <c r="C143" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="D143" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E143" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -3445,13 +3989,16 @@
         <v>143</v>
       </c>
       <c r="C144" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="D144" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E144" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
@@ -3459,13 +4006,16 @@
         <v>144</v>
       </c>
       <c r="C145" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="D145" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E145" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
@@ -3473,13 +4023,16 @@
         <v>145</v>
       </c>
       <c r="C146" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="D146" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E146" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
@@ -3487,13 +4040,16 @@
         <v>146</v>
       </c>
       <c r="C147" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="D147" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E147" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>147</v>
       </c>
@@ -3501,13 +4057,16 @@
         <v>147</v>
       </c>
       <c r="C148" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="D148" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E148" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
@@ -3515,13 +4074,16 @@
         <v>148</v>
       </c>
       <c r="C149" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="D149" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E149" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
@@ -3529,13 +4091,16 @@
         <v>149</v>
       </c>
       <c r="C150" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="D150" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E150" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
       </c>
@@ -3543,13 +4108,16 @@
         <v>150</v>
       </c>
       <c r="C151" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="D151" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E151" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>151</v>
       </c>
@@ -3557,13 +4125,16 @@
         <v>151</v>
       </c>
       <c r="C152" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="D152" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E152" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>152</v>
       </c>
@@ -3571,13 +4142,16 @@
         <v>152</v>
       </c>
       <c r="C153" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="D153" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E153" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>153</v>
       </c>
@@ -3585,13 +4159,16 @@
         <v>153</v>
       </c>
       <c r="C154" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="D154" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E154" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>154</v>
       </c>
@@ -3599,13 +4176,16 @@
         <v>154</v>
       </c>
       <c r="C155" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="D155" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E155" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>155</v>
       </c>
@@ -3613,13 +4193,16 @@
         <v>155</v>
       </c>
       <c r="C156" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="D156" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E156" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>156</v>
       </c>
@@ -3627,13 +4210,16 @@
         <v>156</v>
       </c>
       <c r="C157" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="D157" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E157" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>157</v>
       </c>
@@ -3641,13 +4227,16 @@
         <v>157</v>
       </c>
       <c r="C158" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="D158" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E158" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>158</v>
       </c>
@@ -3655,13 +4244,16 @@
         <v>158</v>
       </c>
       <c r="C159" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="D159" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E159" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>159</v>
       </c>
@@ -3669,13 +4261,16 @@
         <v>159</v>
       </c>
       <c r="C160" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="D160" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E160" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>160</v>
       </c>
@@ -3683,13 +4278,16 @@
         <v>160</v>
       </c>
       <c r="C161" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="D161" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E161" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>161</v>
       </c>
@@ -3697,13 +4295,16 @@
         <v>161</v>
       </c>
       <c r="C162" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="D162" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E162" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>162</v>
       </c>
@@ -3711,13 +4312,16 @@
         <v>162</v>
       </c>
       <c r="C163" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="D163" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+      <c r="E163" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>163</v>
       </c>
@@ -3725,13 +4329,16 @@
         <v>163</v>
       </c>
       <c r="C164" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="D164" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E164" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>164</v>
       </c>
@@ -3739,13 +4346,16 @@
         <v>164</v>
       </c>
       <c r="C165" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="D165" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E165" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>165</v>
       </c>
@@ -3753,13 +4363,16 @@
         <v>165</v>
       </c>
       <c r="C166" t="s">
-        <v>143</v>
+        <v>168</v>
       </c>
       <c r="D166" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E166" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>166</v>
       </c>
@@ -3767,13 +4380,16 @@
         <v>166</v>
       </c>
       <c r="C167" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="D167" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E167" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>167</v>
       </c>
@@ -3781,13 +4397,16 @@
         <v>167</v>
       </c>
       <c r="C168" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="D168" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E168" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>168</v>
       </c>
@@ -3795,13 +4414,16 @@
         <v>168</v>
       </c>
       <c r="C169" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
       <c r="D169" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E169" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>169</v>
       </c>
@@ -3809,13 +4431,16 @@
         <v>169</v>
       </c>
       <c r="C170" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="D170" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E170" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>170</v>
       </c>
@@ -3823,13 +4448,16 @@
         <v>170</v>
       </c>
       <c r="C171" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="D171" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E171" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>171</v>
       </c>
@@ -3837,13 +4465,16 @@
         <v>171</v>
       </c>
       <c r="C172" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="D172" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E172" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>172</v>
       </c>
@@ -3851,13 +4482,16 @@
         <v>172</v>
       </c>
       <c r="C173" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="D173" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E173" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>173</v>
       </c>
@@ -3865,13 +4499,16 @@
         <v>173</v>
       </c>
       <c r="C174" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="D174" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E174" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>174</v>
       </c>
@@ -3879,13 +4516,16 @@
         <v>174</v>
       </c>
       <c r="C175" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="D175" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E175" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>175</v>
       </c>
@@ -3893,13 +4533,16 @@
         <v>175</v>
       </c>
       <c r="C176" t="s">
-        <v>153</v>
+        <v>180</v>
       </c>
       <c r="D176" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E176" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>176</v>
       </c>
@@ -3907,13 +4550,16 @@
         <v>176</v>
       </c>
       <c r="C177" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="D177" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E177" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>177</v>
       </c>
@@ -3921,13 +4567,16 @@
         <v>177</v>
       </c>
       <c r="C178" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="D178" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E178" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>178</v>
       </c>
@@ -3935,13 +4584,16 @@
         <v>178</v>
       </c>
       <c r="C179" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="D179" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E179" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>179</v>
       </c>
@@ -3949,13 +4601,16 @@
         <v>179</v>
       </c>
       <c r="C180" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="D180" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="E180" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>180</v>
       </c>
@@ -3963,13 +4618,16 @@
         <v>180</v>
       </c>
       <c r="C181" t="s">
-        <v>158</v>
+        <v>185</v>
       </c>
       <c r="D181" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E181" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>181</v>
       </c>
@@ -3977,13 +4635,16 @@
         <v>181</v>
       </c>
       <c r="C182" t="s">
-        <v>159</v>
+        <v>187</v>
       </c>
       <c r="D182" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E182" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>182</v>
       </c>
@@ -3991,13 +4652,16 @@
         <v>182</v>
       </c>
       <c r="C183" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
       <c r="D183" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E183" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>183</v>
       </c>
@@ -4005,13 +4669,16 @@
         <v>183</v>
       </c>
       <c r="C184" t="s">
-        <v>161</v>
+        <v>190</v>
       </c>
       <c r="D184" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E184" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>184</v>
       </c>
@@ -4019,13 +4686,16 @@
         <v>184</v>
       </c>
       <c r="C185" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="D185" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E185" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>185</v>
       </c>
@@ -4033,13 +4703,16 @@
         <v>185</v>
       </c>
       <c r="C186" t="s">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="D186" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E186" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>186</v>
       </c>
@@ -4047,13 +4720,16 @@
         <v>186</v>
       </c>
       <c r="C187" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="D187" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E187" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>187</v>
       </c>
@@ -4061,13 +4737,16 @@
         <v>187</v>
       </c>
       <c r="C188" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="D188" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E188" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>188</v>
       </c>
@@ -4075,13 +4754,16 @@
         <v>188</v>
       </c>
       <c r="C189" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="D189" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E189" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>189</v>
       </c>
@@ -4089,13 +4771,16 @@
         <v>189</v>
       </c>
       <c r="C190" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="D190" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E190" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>190</v>
       </c>
@@ -4103,13 +4788,19 @@
         <v>190</v>
       </c>
       <c r="C191" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="D191" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F191" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>191</v>
       </c>
@@ -4117,13 +4808,16 @@
         <v>191</v>
       </c>
       <c r="C192" t="s">
-        <v>165</v>
+        <v>196</v>
       </c>
       <c r="D192" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E192" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>192</v>
       </c>
@@ -4131,13 +4825,16 @@
         <v>192</v>
       </c>
       <c r="C193" t="s">
-        <v>166</v>
+        <v>197</v>
       </c>
       <c r="D193" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E193" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>193</v>
       </c>
@@ -4145,13 +4842,16 @@
         <v>193</v>
       </c>
       <c r="C194" t="s">
-        <v>167</v>
+        <v>198</v>
       </c>
       <c r="D194" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="E194" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>194</v>
       </c>
@@ -4159,13 +4859,16 @@
         <v>194</v>
       </c>
       <c r="C195" t="s">
-        <v>168</v>
+        <v>199</v>
       </c>
       <c r="D195" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="E195" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>195</v>
       </c>
@@ -4173,24 +4876,13 @@
         <v>195</v>
       </c>
       <c r="C196" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="D196" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A197">
-        <v>196</v>
-      </c>
-      <c r="B197">
-        <v>196</v>
-      </c>
-      <c r="C197" t="s">
-        <v>170</v>
-      </c>
-      <c r="D197" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="E196" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to PRo project gdb files to map BESE and grid cases.
</commit_message>
<xml_diff>
--- a/output_tables/group_summary.xlsx
+++ b/output_tables/group_summary.xlsx
@@ -1,26 +1,61 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{59E47FFB-B8F7-45C3-A319-0743BC9995C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF9EF313-13FD-43B7-83F0-2D6B6F9A5433}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="8_{59E47FFB-B8F7-45C3-A319-0743BC9995C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D408E0AB-9DF9-AD4A-A103-5682F61C64C9}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="240" windowWidth="24405" windowHeight="15390" xr2:uid="{DE4F24FA-FBA3-478C-9F9E-E001BBB69A88}"/>
+    <workbookView xWindow="20" yWindow="600" windowWidth="35360" windowHeight="21440" xr2:uid="{DE4F24FA-FBA3-478C-9F9E-E001BBB69A88}"/>
   </bookViews>
   <sheets>
     <sheet name="group_summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">group_summary!$E$1:$E$196</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="0">group_summary!$I$4</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={6A90BB48-253F-4548-8CCC-E8AD25415F61}</author>
+  </authors>
+  <commentList>
+    <comment ref="F89" authorId="0" shapeId="0" xr:uid="{6A90BB48-253F-4548-8CCC-E8AD25415F61}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This was resolved by manually editing the activity_filter in the snapshot input data so that BESE plantings were distinct.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="233">
   <si>
     <t>group_no</t>
   </si>
@@ -638,13 +673,94 @@
   </si>
   <si>
     <t>Is this a mix of donor plants from the other co-located cases?</t>
+  </si>
+  <si>
+    <t>group count</t>
+  </si>
+  <si>
+    <t>total count</t>
+  </si>
+  <si>
+    <t>mixed donor count</t>
+  </si>
+  <si>
+    <t>DPW</t>
+  </si>
+  <si>
+    <t>RKB</t>
+  </si>
+  <si>
+    <t>DMB</t>
+  </si>
+  <si>
+    <t>WNB</t>
+  </si>
+  <si>
+    <t>CTI</t>
+  </si>
+  <si>
+    <t>KTI</t>
+  </si>
+  <si>
+    <t>FYB</t>
+  </si>
+  <si>
+    <t>SNH</t>
+  </si>
+  <si>
+    <t>MTB</t>
+  </si>
+  <si>
+    <t>THC</t>
+  </si>
+  <si>
+    <t>PTJ</t>
+  </si>
+  <si>
+    <t>QLB</t>
+  </si>
+  <si>
+    <t>SPT</t>
+  </si>
+  <si>
+    <t>AND</t>
+  </si>
+  <si>
+    <t>CPT</t>
+  </si>
+  <si>
+    <t>SKB</t>
+  </si>
+  <si>
+    <t>FWB</t>
+  </si>
+  <si>
+    <t>SHH</t>
+  </si>
+  <si>
+    <t>PNT</t>
+  </si>
+  <si>
+    <t>GPT</t>
+  </si>
+  <si>
+    <t>RPT</t>
+  </si>
+  <si>
+    <t>BPT</t>
+  </si>
+  <si>
+    <t>Stuart Island</t>
+  </si>
+  <si>
+    <t>SHB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -779,8 +895,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -972,8 +1094,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1103,6 +1231,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1148,10 +1285,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1208,6 +1348,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="DOWTY, PETER (DNR)" id="{750E6FC1-6785-B14C-B0F3-55122449730F}" userId="S::peter.dowty@dnr.wa.gov::01cf875a-4e15-4928-8f93-7a0dfa1efb6b" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1525,20 +1671,31 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="F89" dT="2026-05-18T04:56:28.25" personId="{750E6FC1-6785-B14C-B0F3-55122449730F}" id="{6A90BB48-253F-4548-8CCC-E8AD25415F61}">
+    <text>This was resolved by manually editing the activity_filter in the snapshot input data so that BESE plantings were distinct.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4FED8F-716B-4B06-A141-CFC261A1ADE2}">
-  <dimension ref="A1:F196"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4FED8F-716B-4B06-A141-CFC261A1ADE2}">
+  <dimension ref="A1:M196"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="106.85546875" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="106.83203125" customWidth="1"/>
+    <col min="7" max="7" width="2.83203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="31.5" customWidth="1"/>
+    <col min="10" max="10" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1552,7 +1709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1569,7 +1726,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1586,7 +1743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1602,8 +1759,14 @@
       <c r="E4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1619,8 +1782,17 @@
       <c r="E5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5">
+        <v>49</v>
+      </c>
+      <c r="K5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1636,8 +1808,24 @@
       <c r="E6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>210</v>
+      </c>
+      <c r="L6">
+        <f>SUM(J5:J33)</f>
+        <v>195</v>
+      </c>
+      <c r="M6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1653,8 +1841,17 @@
       <c r="E7" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7">
+        <v>19</v>
+      </c>
+      <c r="K7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1670,8 +1867,24 @@
       <c r="E8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J8">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s">
+        <v>218</v>
+      </c>
+      <c r="L8">
+        <f>SUM(J29:J33)</f>
+        <v>10</v>
+      </c>
+      <c r="M8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1687,8 +1900,21 @@
       <c r="E9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9">
+        <v>11</v>
+      </c>
+      <c r="K9" t="s">
+        <v>212</v>
+      </c>
+      <c r="L9" s="5">
+        <f>L8/L6</f>
+        <v>5.128205128205128E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1704,8 +1930,17 @@
       <c r="E10" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>144</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1721,8 +1956,17 @@
       <c r="E11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I11" t="s">
+        <v>166</v>
+      </c>
+      <c r="J11">
+        <v>10</v>
+      </c>
+      <c r="K11" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1738,8 +1982,17 @@
       <c r="E12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1755,8 +2008,17 @@
       <c r="E13" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
+      <c r="K13" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1772,8 +2034,17 @@
       <c r="E14" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14">
+        <v>6</v>
+      </c>
+      <c r="K14" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1789,8 +2060,17 @@
       <c r="E15" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>45</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1806,8 +2086,17 @@
       <c r="E16" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>179</v>
+      </c>
+      <c r="J16">
+        <v>4</v>
+      </c>
+      <c r="K16" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1823,8 +2112,17 @@
       <c r="E17" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I17" t="s">
+        <v>9</v>
+      </c>
+      <c r="J17">
+        <v>3</v>
+      </c>
+      <c r="K17" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1840,8 +2138,17 @@
       <c r="E18" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>33</v>
+      </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
+      <c r="K18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1857,8 +2164,17 @@
       <c r="E19" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>32</v>
+      </c>
+      <c r="J19">
+        <v>2</v>
+      </c>
+      <c r="K19" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1874,8 +2190,17 @@
       <c r="E20" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>34</v>
+      </c>
+      <c r="J20">
+        <v>2</v>
+      </c>
+      <c r="K20" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1891,8 +2216,17 @@
       <c r="E21" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>64</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="K21" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1908,8 +2242,17 @@
       <c r="E22" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I22" t="s">
+        <v>120</v>
+      </c>
+      <c r="J22">
+        <v>2</v>
+      </c>
+      <c r="K22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1928,8 +2271,17 @@
       <c r="F23" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I23" t="s">
+        <v>186</v>
+      </c>
+      <c r="J23">
+        <v>2</v>
+      </c>
+      <c r="K23" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1945,8 +2297,17 @@
       <c r="E24" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I24" t="s">
+        <v>52</v>
+      </c>
+      <c r="J24">
+        <v>1</v>
+      </c>
+      <c r="K24" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1962,8 +2323,17 @@
       <c r="E25" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I25" t="s">
+        <v>76</v>
+      </c>
+      <c r="J25">
+        <v>1</v>
+      </c>
+      <c r="K25" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1979,8 +2349,17 @@
       <c r="E26" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I26" t="s">
+        <v>177</v>
+      </c>
+      <c r="J26">
+        <v>1</v>
+      </c>
+      <c r="K26" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1996,8 +2375,17 @@
       <c r="E27" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I27" t="s">
+        <v>191</v>
+      </c>
+      <c r="J27">
+        <v>1</v>
+      </c>
+      <c r="K27" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2013,8 +2401,17 @@
       <c r="E28" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I28" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="J28" s="4">
+        <v>1</v>
+      </c>
+      <c r="K28" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2030,8 +2427,14 @@
       <c r="E29" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I29" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="J29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2047,8 +2450,14 @@
       <c r="E30" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2064,8 +2473,14 @@
       <c r="E31" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2081,8 +2496,14 @@
       <c r="E32" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I32" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2098,8 +2519,14 @@
       <c r="E33" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I33" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2116,7 +2543,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2132,8 +2559,14 @@
       <c r="E35" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="I35" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="K35" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2150,7 +2583,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2167,7 +2600,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2184,7 +2617,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2201,7 +2634,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2218,7 +2651,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2235,7 +2668,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2252,7 +2685,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2269,7 +2702,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2286,7 +2719,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2303,7 +2736,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2320,7 +2753,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2337,7 +2770,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2354,7 +2787,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2371,7 +2804,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2388,7 +2821,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2405,7 +2838,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2422,7 +2855,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2439,7 +2872,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2456,7 +2889,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2473,7 +2906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2490,7 +2923,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2507,7 +2940,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2524,7 +2957,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2541,7 +2974,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2558,7 +2991,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2575,7 +3008,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2592,7 +3025,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2609,7 +3042,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2626,7 +3059,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2643,7 +3076,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2660,7 +3093,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2677,7 +3110,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2694,7 +3127,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2711,7 +3144,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2728,7 +3161,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2745,7 +3178,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2762,7 +3195,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2779,7 +3212,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2796,7 +3229,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2813,7 +3246,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2830,7 +3263,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2847,7 +3280,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2864,7 +3297,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2881,7 +3314,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2898,7 +3331,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2915,7 +3348,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2932,7 +3365,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2949,7 +3382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2966,7 +3399,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2983,7 +3416,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -3000,7 +3433,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -3017,7 +3450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3034,7 +3467,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3054,7 +3487,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3074,7 +3507,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3094,7 +3527,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3114,7 +3547,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -3131,7 +3564,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3148,7 +3581,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3165,7 +3598,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3182,7 +3615,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3199,7 +3632,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3216,7 +3649,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3233,7 +3666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3250,7 +3683,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3267,7 +3700,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3284,7 +3717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3301,7 +3734,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3318,7 +3751,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3335,7 +3768,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3352,7 +3785,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3369,7 +3802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3386,7 +3819,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3403,7 +3836,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3420,7 +3853,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3437,7 +3870,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3454,7 +3887,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3471,7 +3904,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3488,7 +3921,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3505,7 +3938,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3522,7 +3955,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3539,7 +3972,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3556,7 +3989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>118</v>
       </c>
@@ -3573,7 +4006,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>119</v>
       </c>
@@ -3590,7 +4023,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>120</v>
       </c>
@@ -3607,7 +4040,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3624,7 +4057,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3641,7 +4074,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3658,7 +4091,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3675,7 +4108,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3692,7 +4125,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3709,7 +4142,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3726,7 +4159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3743,7 +4176,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3760,7 +4193,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3777,7 +4210,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>131</v>
       </c>
@@ -3794,7 +4227,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>132</v>
       </c>
@@ -3811,7 +4244,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>133</v>
       </c>
@@ -3828,7 +4261,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>134</v>
       </c>
@@ -3845,7 +4278,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>135</v>
       </c>
@@ -3862,7 +4295,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>136</v>
       </c>
@@ -3879,7 +4312,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>137</v>
       </c>
@@ -3896,7 +4329,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>138</v>
       </c>
@@ -3913,7 +4346,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>139</v>
       </c>
@@ -3930,7 +4363,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>140</v>
       </c>
@@ -3947,7 +4380,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>141</v>
       </c>
@@ -3964,7 +4397,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>142</v>
       </c>
@@ -3981,7 +4414,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>143</v>
       </c>
@@ -3998,7 +4431,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>144</v>
       </c>
@@ -4015,7 +4448,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>145</v>
       </c>
@@ -4032,7 +4465,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>146</v>
       </c>
@@ -4049,7 +4482,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>147</v>
       </c>
@@ -4066,7 +4499,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>148</v>
       </c>
@@ -4083,7 +4516,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>149</v>
       </c>
@@ -4100,7 +4533,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>150</v>
       </c>
@@ -4117,7 +4550,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>151</v>
       </c>
@@ -4134,7 +4567,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>152</v>
       </c>
@@ -4151,7 +4584,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>153</v>
       </c>
@@ -4168,7 +4601,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>154</v>
       </c>
@@ -4185,7 +4618,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>155</v>
       </c>
@@ -4202,7 +4635,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>156</v>
       </c>
@@ -4219,7 +4652,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>157</v>
       </c>
@@ -4236,7 +4669,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>158</v>
       </c>
@@ -4253,7 +4686,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>159</v>
       </c>
@@ -4270,7 +4703,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>160</v>
       </c>
@@ -4287,7 +4720,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>161</v>
       </c>
@@ -4304,7 +4737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>162</v>
       </c>
@@ -4321,7 +4754,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>163</v>
       </c>
@@ -4338,7 +4771,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>164</v>
       </c>
@@ -4355,7 +4788,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>165</v>
       </c>
@@ -4372,7 +4805,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>166</v>
       </c>
@@ -4389,7 +4822,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>167</v>
       </c>
@@ -4406,7 +4839,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>168</v>
       </c>
@@ -4423,7 +4856,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>169</v>
       </c>
@@ -4440,7 +4873,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>170</v>
       </c>
@@ -4457,7 +4890,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>171</v>
       </c>
@@ -4474,7 +4907,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>172</v>
       </c>
@@ -4491,7 +4924,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>173</v>
       </c>
@@ -4508,7 +4941,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>174</v>
       </c>
@@ -4525,7 +4958,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>175</v>
       </c>
@@ -4542,7 +4975,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>176</v>
       </c>
@@ -4559,7 +4992,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>177</v>
       </c>
@@ -4576,7 +5009,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>178</v>
       </c>
@@ -4593,7 +5026,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>179</v>
       </c>
@@ -4610,7 +5043,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>180</v>
       </c>
@@ -4627,7 +5060,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>181</v>
       </c>
@@ -4644,7 +5077,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>182</v>
       </c>
@@ -4661,7 +5094,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>183</v>
       </c>
@@ -4678,7 +5111,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>184</v>
       </c>
@@ -4695,7 +5128,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>185</v>
       </c>
@@ -4712,7 +5145,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>186</v>
       </c>
@@ -4729,7 +5162,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>187</v>
       </c>
@@ -4746,7 +5179,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>188</v>
       </c>
@@ -4763,7 +5196,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>189</v>
       </c>
@@ -4780,7 +5213,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>190</v>
       </c>
@@ -4800,7 +5233,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>191</v>
       </c>
@@ -4817,7 +5250,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>192</v>
       </c>
@@ -4834,7 +5267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>193</v>
       </c>
@@ -4851,7 +5284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>194</v>
       </c>
@@ -4868,7 +5301,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>195</v>
       </c>
@@ -4886,7 +5319,11 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I5:J29">
+    <sortCondition descending="1" ref="J5:J29"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>